<commit_message>
Update BOM spreadsheet and Suntracker PDF
Replace BOM/BOM.xlsx and Documentation/Suntracker.pdf with updated binary versions. The spreadsheet updates the bill of materials and the PDF refreshes the Suntracker documentation; no source code changes.
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12300"/>
+    <workbookView windowWidth="27945" windowHeight="11700" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Elektronic" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="109">
   <si>
     <t>Reference</t>
   </si>
@@ -352,6 +352,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>GT2 belt 220 mm</t>
   </si>
 </sst>
 </file>
@@ -982,7 +985,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -992,11 +995,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2097,7 +2103,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="40.1428571428571" customWidth="1"/>
@@ -2192,11 +2198,19 @@
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>